<commit_message>
chore: import nist-100-1/schema/nist-ai-rmf-common schema
</commit_message>
<xml_diff>
--- a/project/excel/nist_ai_600_1.xlsx
+++ b/project/excel/nist_ai_600_1.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,19 +449,19 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>trustworthiness_characteristic</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>addressed_by_actions</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>lifecycle_stage</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>trustworthiness_characteristic</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>addressed_by_actions</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
         <is>
           <t>id</t>
@@ -469,12 +469,22 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>description</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>see_also</t>
         </is>
       </c>
     </row>
@@ -493,10 +503,10 @@
       <formula1>"IMMEDIATE,PROLONGED"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"VALID_AND_RELIABLE,SAFE,SECURE_AND_RESILIENT,ACCOUNTABLE_AND_TRANSPARENT,EXPLAINABLE_AND_INTERPRETABLE,PRIVACY_ENHANCED,FAIR_WITH_HARMFUL_BIAS_MANAGED"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"DESIGN,DEVELOPMENT,DEPLOYMENT,OPERATION,DECOMMISSIONING"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"VALID_AND_RELIABLE,SAFE,SECURE_AND_RESILIENT,ACCOUNTABLE_AND_TRANSPARENT,EXPLAINABLE_AND_INTERPRETABLE,PRIVACY_ENHANCED,FAIR_WITH_HARMFUL_BIAS_MANAGED"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -509,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,12 +555,22 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>description</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>see_also</t>
         </is>
       </c>
     </row>
@@ -573,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -614,12 +634,22 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>description</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>see_also</t>
         </is>
       </c>
     </row>
@@ -642,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -658,12 +688,22 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>description</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>see_also</t>
         </is>
       </c>
     </row>
@@ -683,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -704,12 +744,22 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>see_also</t>
         </is>
       </c>
     </row>
@@ -732,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -763,12 +813,22 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>description</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>see_also</t>
         </is>
       </c>
     </row>

</xml_diff>